<commit_message>
Organization types: School, Company, Organization, Ministry... picked on New customer, customer profile and website sign-up; a customer's screens say its word instead of "school" in every language
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/NTCSWEB-Modules.xlsx
+++ b/docs/NTCSWEB-Modules.xlsx
@@ -643,7 +643,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K39"/>
+  <dimension ref="A1:K40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2082,6 +2082,51 @@
       <c r="K39" s="18" t="inlineStr">
         <is>
           <t>Own password and two-factor sign-in (profile row at the bottom of the menu).</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="21.6" customHeight="1">
+      <c r="A40" s="1" t="inlineStr">
+        <is>
+          <t>A11</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Organization types</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>ប្រភេទស្ថាប័ន</t>
+        </is>
+      </c>
+      <c r="D40" s="1" t="inlineStr">
+        <is>
+          <t>A11.1</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>Organization types</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>ប្រភេទស្ថាប័ន</t>
+        </is>
+      </c>
+      <c r="G40" s="4" t="inlineStr">
+        <is>
+          <t>/organization-types</t>
+        </is>
+      </c>
+      <c r="H40" s="5" t="n"/>
+      <c r="I40" s="3" t="n"/>
+      <c r="J40" s="3" t="n"/>
+      <c r="K40" s="6" t="inlineStr">
+        <is>
+          <t>In the menu right under Customers. School, Company, Organization, Ministry… with their word for "school" in each language; a customer's screens use its word. Picked on New customer, the customer profile and website sign-up.</t>
         </is>
       </c>
     </row>

</xml_diff>